<commit_message>
Update economic data 2026-04-13
</commit_message>
<xml_diff>
--- a/data/長期系列_CI指数_DI指数_DI景気指標.xlsx
+++ b/data/長期系列_CI指数_DI指数_DI景気指標.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\CI\０１／CI\０２／速報からの改訂\★R8(2026)★\令和8年1月改訂\g研究所ホームページ掲載宛送付ファイル\jp\stat\di\di\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\CI\０１／CI\０１／速報\★R8(2026)★\令和8年2月分\g研究所ホームページ掲載宛送付ファイル\jp\stat\di\di\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{73340567-A5C6-4B12-B2F2-A445F1E58F8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{44BC624A-4D4C-404B-99D2-5C917448A2F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="619" uniqueCount="577">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="578">
   <si>
     <t>ＤＩ指数</t>
   </si>
@@ -2334,6 +2334,10 @@
   </si>
   <si>
     <t>2026000101</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>2026000202</t>
     <phoneticPr fontId="2"/>
   </si>
 </sst>
@@ -2835,7 +2839,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P568"/>
+  <dimension ref="A1:P569"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.6640625" bestFit="1" customWidth="1"/>
@@ -28271,7 +28275,7 @@
         <v>12</v>
       </c>
       <c r="D558" s="4">
-        <v>110.4</v>
+        <v>110.5</v>
       </c>
       <c r="E558" s="4">
         <v>114.5</v>
@@ -28354,13 +28358,60 @@
         <v>3178</v>
       </c>
     </row>
-    <row r="568" spans="4:9" x14ac:dyDescent="0.2">
-      <c r="D568" s="3"/>
-      <c r="E568" s="3"/>
-      <c r="F568" s="3"/>
-      <c r="G568" s="3"/>
-      <c r="H568" s="3"/>
-      <c r="I568" s="3"/>
+    <row r="560" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A560" s="13" t="s">
+        <v>577</v>
+      </c>
+      <c r="B560" s="2">
+        <v>2026</v>
+      </c>
+      <c r="C560" s="2">
+        <v>2</v>
+      </c>
+      <c r="D560" s="4">
+        <v>112.4</v>
+      </c>
+      <c r="E560" s="4">
+        <v>116.3</v>
+      </c>
+      <c r="F560" s="4">
+        <v>112.2</v>
+      </c>
+      <c r="G560" s="4">
+        <v>112.1</v>
+      </c>
+      <c r="H560" s="4">
+        <v>114.2</v>
+      </c>
+      <c r="I560" s="4">
+        <v>108.5</v>
+      </c>
+      <c r="J560" s="4">
+        <v>72.2</v>
+      </c>
+      <c r="K560" s="4">
+        <v>68.8</v>
+      </c>
+      <c r="L560" s="4">
+        <v>50</v>
+      </c>
+      <c r="M560" s="4">
+        <v>1323.9</v>
+      </c>
+      <c r="N560" s="4">
+        <v>3241.6</v>
+      </c>
+      <c r="O560" s="4">
+        <v>3178</v>
+      </c>
+    </row>
+    <row r="569" spans="4:9" x14ac:dyDescent="0.2">
+      <c r="D569" s="3"/>
+      <c r="E569" s="3"/>
+      <c r="F569" s="3"/>
+      <c r="G569" s="3"/>
+      <c r="H569" s="3"/>
+      <c r="I569" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2"/>

</xml_diff>

<commit_message>
Update economic data 2026-06-29
</commit_message>
<xml_diff>
--- a/data/長期系列_CI指数_DI指数_DI景気指標.xlsx
+++ b/data/長期系列_CI指数_DI指数_DI景気指標.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\CI\０１／CI\０１／速報\★R8(2026)★\令和8年4月分\g研究所ホームページ掲載宛送付ファイル\jp\stat\di\di\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\CI\０１／CI\０２／速報からの改訂\★R8(2026)★\令和8年4月改訂\g研究所ホームページ掲載宛送付ファイル\jp\stat\di\di\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9EB14EED-CD0E-47F2-9D3D-013214BA9F19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AC65CF96-2660-4183-936C-743DEF0B68C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456"/>
   </bookViews>
@@ -28345,7 +28345,7 @@
         <v>115.6</v>
       </c>
       <c r="I559" s="4">
-        <v>108.9</v>
+        <v>108.8</v>
       </c>
       <c r="J559" s="4">
         <v>77.3</v>
@@ -28471,40 +28471,40 @@
         <v>4</v>
       </c>
       <c r="D562" s="4">
-        <v>115.9</v>
+        <v>116.1</v>
       </c>
       <c r="E562" s="4">
-        <v>117.9</v>
+        <v>118.1</v>
       </c>
       <c r="F562" s="4">
-        <v>111.2</v>
+        <v>111.9</v>
       </c>
       <c r="G562" s="4">
-        <v>113.6</v>
+        <v>113.8</v>
       </c>
       <c r="H562" s="4">
-        <v>115.6</v>
+        <v>115.8</v>
       </c>
       <c r="I562" s="4">
-        <v>107.7</v>
+        <v>108.5</v>
       </c>
       <c r="J562" s="4">
-        <v>44.4</v>
+        <v>50</v>
       </c>
       <c r="K562" s="4">
-        <v>43.8</v>
+        <v>50</v>
       </c>
       <c r="L562" s="4">
-        <v>50</v>
+        <v>37.5</v>
       </c>
       <c r="M562" s="4">
-        <v>1371.1</v>
+        <v>1376.7</v>
       </c>
       <c r="N562" s="4">
-        <v>3268.8</v>
+        <v>3275</v>
       </c>
       <c r="O562" s="4">
-        <v>3123.8</v>
+        <v>3111.3</v>
       </c>
     </row>
     <row r="571" spans="1:15" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Update economic data 2026-07-13
</commit_message>
<xml_diff>
--- a/data/長期系列_CI指数_DI指数_DI景気指標.xlsx
+++ b/data/長期系列_CI指数_DI指数_DI景気指標.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\CI\０１／CI\０２／速報からの改訂\★R8(2026)★\令和8年4月改訂\g研究所ホームページ掲載宛送付ファイル\jp\stat\di\di\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\CI\０１／CI\０１／速報\★R8(2026)★\令和8年5月分\g研究所ホームページ掲載宛送付ファイル\jp\stat\di\di\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AC65CF96-2660-4183-936C-743DEF0B68C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D117CB5F-3AEB-4CEC-91D7-CA36179D54F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="622" uniqueCount="580">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="623" uniqueCount="581">
   <si>
     <t>ＤＩ指数</t>
   </si>
@@ -2346,6 +2346,10 @@
   </si>
   <si>
     <t>2026000404</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>2026000505</t>
     <phoneticPr fontId="2"/>
   </si>
 </sst>
@@ -2847,7 +2851,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P571"/>
+  <dimension ref="A1:P572"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.6640625" bestFit="1" customWidth="1"/>
@@ -28480,7 +28484,7 @@
         <v>111.9</v>
       </c>
       <c r="G562" s="4">
-        <v>113.8</v>
+        <v>113.7</v>
       </c>
       <c r="H562" s="4">
         <v>115.8</v>
@@ -28507,13 +28511,60 @@
         <v>3111.3</v>
       </c>
     </row>
-    <row r="571" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="D571" s="3"/>
-      <c r="E571" s="3"/>
-      <c r="F571" s="3"/>
-      <c r="G571" s="3"/>
-      <c r="H571" s="3"/>
-      <c r="I571" s="3"/>
+    <row r="563" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A563" s="13" t="s">
+        <v>580</v>
+      </c>
+      <c r="B563" s="2">
+        <v>2026</v>
+      </c>
+      <c r="C563" s="2">
+        <v>5</v>
+      </c>
+      <c r="D563" s="4">
+        <v>116.8</v>
+      </c>
+      <c r="E563" s="4">
+        <v>118.5</v>
+      </c>
+      <c r="F563" s="4">
+        <v>111.5</v>
+      </c>
+      <c r="G563" s="4">
+        <v>114.5</v>
+      </c>
+      <c r="H563" s="4">
+        <v>116.1</v>
+      </c>
+      <c r="I563" s="4">
+        <v>108.1</v>
+      </c>
+      <c r="J563" s="4">
+        <v>55.6</v>
+      </c>
+      <c r="K563" s="4">
+        <v>75</v>
+      </c>
+      <c r="L563" s="4">
+        <v>33.299999999999997</v>
+      </c>
+      <c r="M563" s="4">
+        <v>1382.3</v>
+      </c>
+      <c r="N563" s="4">
+        <v>3300</v>
+      </c>
+      <c r="O563" s="4">
+        <v>3094.6</v>
+      </c>
+    </row>
+    <row r="572" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="D572" s="3"/>
+      <c r="E572" s="3"/>
+      <c r="F572" s="3"/>
+      <c r="G572" s="3"/>
+      <c r="H572" s="3"/>
+      <c r="I572" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2"/>

</xml_diff>

<commit_message>
Update economic data 2026-07-27
</commit_message>
<xml_diff>
--- a/data/長期系列_CI指数_DI指数_DI景気指標.xlsx
+++ b/data/長期系列_CI指数_DI指数_DI景気指標.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\CI\０１／CI\０１／速報\★R8(2026)★\令和8年5月分\g研究所ホームページ掲載宛送付ファイル\jp\stat\di\di\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\CI\０１／CI\０２／速報からの改訂\★R8(2026)★\令和8年5月改訂\g研究所ホームページ掲載宛送付ファイル\jp\stat\di\di\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D117CB5F-3AEB-4CEC-91D7-CA36179D54F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0F215A26-7662-4B13-939A-B0681FDFC4A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{91D94BF3-D2EC-4E14-92C7-563E09D9EA03}"/>
   </bookViews>
   <sheets>
     <sheet name="指数 Indexes" sheetId="1" r:id="rId1"/>
@@ -25,6 +25,8 @@
         <xcalcf:feature name="microsoft.com:RD"/>
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
@@ -2356,7 +2358,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="179" formatCode="0.0_);[Red]\(0.0\)"/>
     <numFmt numFmtId="207" formatCode="0.0_ ;[Red]\-0.0\ "/>
@@ -2444,7 +2446,7 @@
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
-    <cellStyle name="標準 2" xfId="1"/>
+    <cellStyle name="標準 2" xfId="1" xr:uid="{C0990F8C-84CB-4C08-9886-26AB3DA3BD94}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -2528,9 +2530,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office テーマ">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2568,9 +2570,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -2603,26 +2605,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -2655,26 +2640,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2847,7 +2815,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ACAF9C03-5388-439A-97AC-994DCAA1A5D5}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -28481,7 +28449,7 @@
         <v>118.1</v>
       </c>
       <c r="F562" s="4">
-        <v>111.9</v>
+        <v>111.6</v>
       </c>
       <c r="G562" s="4">
         <v>113.7</v>
@@ -28490,7 +28458,7 @@
         <v>115.8</v>
       </c>
       <c r="I562" s="4">
-        <v>108.5</v>
+        <v>108.4</v>
       </c>
       <c r="J562" s="4">
         <v>50</v>
@@ -28522,40 +28490,40 @@
         <v>5</v>
       </c>
       <c r="D563" s="4">
-        <v>116.8</v>
+        <v>116.5</v>
       </c>
       <c r="E563" s="4">
-        <v>118.5</v>
+        <v>117.9</v>
       </c>
       <c r="F563" s="4">
-        <v>111.5</v>
+        <v>111.4</v>
       </c>
       <c r="G563" s="4">
-        <v>114.5</v>
+        <v>114.1</v>
       </c>
       <c r="H563" s="4">
-        <v>116.1</v>
+        <v>115.5</v>
       </c>
       <c r="I563" s="4">
         <v>108.1</v>
       </c>
       <c r="J563" s="4">
-        <v>55.6</v>
+        <v>60</v>
       </c>
       <c r="K563" s="4">
-        <v>75</v>
+        <v>66.7</v>
       </c>
       <c r="L563" s="4">
-        <v>33.299999999999997</v>
+        <v>50</v>
       </c>
       <c r="M563" s="4">
-        <v>1382.3</v>
+        <v>1386.7</v>
       </c>
       <c r="N563" s="4">
-        <v>3300</v>
+        <v>3291.7</v>
       </c>
       <c r="O563" s="4">
-        <v>3094.6</v>
+        <v>3111.3</v>
       </c>
     </row>
     <row r="572" spans="1:15" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Update economic data 2026-08-09
</commit_message>
<xml_diff>
--- a/data/長期系列_CI指数_DI指数_DI景気指標.xlsx
+++ b/data/長期系列_CI指数_DI指数_DI景気指標.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\CI\０１／CI\０２／速報からの改訂\★R8(2026)★\令和8年5月改訂\g研究所ホームページ掲載宛送付ファイル\jp\stat\di\di\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\CI\０１／CI\０１／速報\★R8(2026)★\令和8年6月分\g研究所ホームページ掲載宛送付ファイル\jp\stat\di\di\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0F215A26-7662-4B13-939A-B0681FDFC4A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FE07788C-AC71-4286-884C-930879EFE0A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{91D94BF3-D2EC-4E14-92C7-563E09D9EA03}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CBAC15B1-C8E8-48BC-A52C-EDC979E563C6}"/>
   </bookViews>
   <sheets>
     <sheet name="指数 Indexes" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="623" uniqueCount="581">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="624" uniqueCount="582">
   <si>
     <t>ＤＩ指数</t>
   </si>
@@ -2352,6 +2352,10 @@
   </si>
   <si>
     <t>2026000505</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>2026000606</t>
     <phoneticPr fontId="2"/>
   </si>
 </sst>
@@ -2446,7 +2450,7 @@
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
-    <cellStyle name="標準 2" xfId="1" xr:uid="{C0990F8C-84CB-4C08-9886-26AB3DA3BD94}"/>
+    <cellStyle name="標準 2" xfId="1" xr:uid="{DD74F69C-CDE4-4E35-9566-348258E22433}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -2815,11 +2819,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ACAF9C03-5388-439A-97AC-994DCAA1A5D5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4E461FE-5748-4EBE-A583-8B039D6E9CA4}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P572"/>
+  <dimension ref="A1:P573"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.6640625" bestFit="1" customWidth="1"/>
@@ -28490,7 +28494,7 @@
         <v>5</v>
       </c>
       <c r="D563" s="4">
-        <v>116.5</v>
+        <v>116.4</v>
       </c>
       <c r="E563" s="4">
         <v>117.9</v>
@@ -28526,13 +28530,60 @@
         <v>3111.3</v>
       </c>
     </row>
-    <row r="572" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="D572" s="3"/>
-      <c r="E572" s="3"/>
-      <c r="F572" s="3"/>
-      <c r="G572" s="3"/>
-      <c r="H572" s="3"/>
-      <c r="I572" s="3"/>
+    <row r="564" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A564" s="13" t="s">
+        <v>581</v>
+      </c>
+      <c r="B564" s="2">
+        <v>2026</v>
+      </c>
+      <c r="C564" s="2">
+        <v>6</v>
+      </c>
+      <c r="D564" s="4">
+        <v>116.4</v>
+      </c>
+      <c r="E564" s="4">
+        <v>118.2</v>
+      </c>
+      <c r="F564" s="4">
+        <v>112.3</v>
+      </c>
+      <c r="G564" s="4">
+        <v>114</v>
+      </c>
+      <c r="H564" s="4">
+        <v>115.9</v>
+      </c>
+      <c r="I564" s="4">
+        <v>108.9</v>
+      </c>
+      <c r="J564" s="4">
+        <v>55.6</v>
+      </c>
+      <c r="K564" s="4">
+        <v>68.8</v>
+      </c>
+      <c r="L564" s="4">
+        <v>50</v>
+      </c>
+      <c r="M564" s="4">
+        <v>1392.3</v>
+      </c>
+      <c r="N564" s="4">
+        <v>3310.5</v>
+      </c>
+      <c r="O564" s="4">
+        <v>3111.3</v>
+      </c>
+    </row>
+    <row r="573" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="D573" s="3"/>
+      <c r="E573" s="3"/>
+      <c r="F573" s="3"/>
+      <c r="G573" s="3"/>
+      <c r="H573" s="3"/>
+      <c r="I573" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2"/>

</xml_diff>

<commit_message>
Update economic data 2026-08-31
</commit_message>
<xml_diff>
--- a/data/長期系列_CI指数_DI指数_DI景気指標.xlsx
+++ b/data/長期系列_CI指数_DI指数_DI景気指標.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\CI\０１／CI\０１／速報\★R8(2026)★\令和8年6月分\g研究所ホームページ掲載宛送付ファイル\jp\stat\di\di\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\CI\０１／CI\０２／速報からの改訂\★R8(2026)★\令和8年6月改訂\g研究所ホームページ掲載宛送付ファイル\jp\stat\di\di\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FE07788C-AC71-4286-884C-930879EFE0A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{751B49AE-11A7-4CEE-A53D-12854C20AF41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CBAC15B1-C8E8-48BC-A52C-EDC979E563C6}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2019AAFD-9813-4CF2-B98C-90438DBBD93A}"/>
   </bookViews>
   <sheets>
     <sheet name="指数 Indexes" sheetId="1" r:id="rId1"/>
@@ -2450,7 +2450,7 @@
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
-    <cellStyle name="標準 2" xfId="1" xr:uid="{DD74F69C-CDE4-4E35-9566-348258E22433}"/>
+    <cellStyle name="標準 2" xfId="1" xr:uid="{5C646276-010B-469B-A671-04CF1791B3BF}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -2819,7 +2819,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4E461FE-5748-4EBE-A583-8B039D6E9CA4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{812EC5AB-4E54-4C5A-ABDF-08F1F40AD455}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -27569,7 +27569,7 @@
         <v>111.9</v>
       </c>
       <c r="I543" s="4">
-        <v>106.6</v>
+        <v>106.7</v>
       </c>
       <c r="J543" s="4">
         <v>45.5</v>
@@ -27710,7 +27710,7 @@
         <v>114.1</v>
       </c>
       <c r="I546" s="4">
-        <v>108</v>
+        <v>107.9</v>
       </c>
       <c r="J546" s="4">
         <v>54.5</v>
@@ -28321,7 +28321,7 @@
         <v>115.6</v>
       </c>
       <c r="I559" s="4">
-        <v>108.8</v>
+        <v>108.7</v>
       </c>
       <c r="J559" s="4">
         <v>77.3</v>
@@ -28368,7 +28368,7 @@
         <v>114.2</v>
       </c>
       <c r="I560" s="4">
-        <v>108.6</v>
+        <v>108.5</v>
       </c>
       <c r="J560" s="4">
         <v>77.3</v>
@@ -28415,7 +28415,7 @@
         <v>114.5</v>
       </c>
       <c r="I561" s="4">
-        <v>108.2</v>
+        <v>108.1</v>
       </c>
       <c r="J561" s="4">
         <v>72.7</v>
@@ -28453,7 +28453,7 @@
         <v>118.1</v>
       </c>
       <c r="F562" s="4">
-        <v>111.6</v>
+        <v>111.7</v>
       </c>
       <c r="G562" s="4">
         <v>113.7</v>
@@ -28494,22 +28494,22 @@
         <v>5</v>
       </c>
       <c r="D563" s="4">
-        <v>116.4</v>
+        <v>116.5</v>
       </c>
       <c r="E563" s="4">
         <v>117.9</v>
       </c>
       <c r="F563" s="4">
-        <v>111.4</v>
+        <v>111.3</v>
       </c>
       <c r="G563" s="4">
-        <v>114.1</v>
+        <v>114.2</v>
       </c>
       <c r="H563" s="4">
         <v>115.5</v>
       </c>
       <c r="I563" s="4">
-        <v>108.1</v>
+        <v>107.9</v>
       </c>
       <c r="J563" s="4">
         <v>60</v>
@@ -28518,7 +28518,7 @@
         <v>66.7</v>
       </c>
       <c r="L563" s="4">
-        <v>50</v>
+        <v>37.5</v>
       </c>
       <c r="M563" s="4">
         <v>1386.7</v>
@@ -28527,7 +28527,7 @@
         <v>3291.7</v>
       </c>
       <c r="O563" s="4">
-        <v>3111.3</v>
+        <v>3098.8</v>
       </c>
     </row>
     <row r="564" spans="1:15" x14ac:dyDescent="0.2">
@@ -28541,40 +28541,40 @@
         <v>6</v>
       </c>
       <c r="D564" s="4">
-        <v>116.4</v>
+        <v>116.5</v>
       </c>
       <c r="E564" s="4">
-        <v>118.2</v>
+        <v>118.5</v>
       </c>
       <c r="F564" s="4">
-        <v>112.3</v>
+        <v>111.8</v>
       </c>
       <c r="G564" s="4">
-        <v>114</v>
+        <v>114.1</v>
       </c>
       <c r="H564" s="4">
-        <v>115.9</v>
+        <v>116.1</v>
       </c>
       <c r="I564" s="4">
-        <v>108.9</v>
+        <v>108.4</v>
       </c>
       <c r="J564" s="4">
-        <v>55.6</v>
+        <v>60</v>
       </c>
       <c r="K564" s="4">
-        <v>68.8</v>
+        <v>72.2</v>
       </c>
       <c r="L564" s="4">
-        <v>50</v>
+        <v>37.5</v>
       </c>
       <c r="M564" s="4">
-        <v>1392.3</v>
+        <v>1396.7</v>
       </c>
       <c r="N564" s="4">
-        <v>3310.5</v>
+        <v>3313.9</v>
       </c>
       <c r="O564" s="4">
-        <v>3111.3</v>
+        <v>3086.3</v>
       </c>
     </row>
     <row r="573" spans="1:15" x14ac:dyDescent="0.2">

</xml_diff>